<commit_message>
Programar corte total 24 h en colegios CORMUP con control.
Deja el Excel de horarios en 00:00-23:59 para los 11 establecimientos con control (desde el domingo 13/09), respalda los horarios nocturnos originales y agrega cormup_corte_total.py más el informe de verificación domingo/lunes.

Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/HORARIOS CONTROL NOCTURNO.xlsx
+++ b/reports/HORARIOS CONTROL NOCTURNO.xlsx
@@ -514,7 +514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:F50"/>
+  <dimension ref="A2:F50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="15.85546875" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -677,7 +677,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 06:00</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 06:00</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>01:00 a 05:59</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 05:59</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 04:00</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F11" s="6" t="inlineStr">
@@ -812,7 +812,7 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 05:59</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -839,7 +839,7 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 05:59</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>01:00 a 05:59</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 05:59</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 05:59</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>00:01 a 05:59</t>
+          <t>00:00 a 23:59</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">

</xml_diff>